<commit_message>
docs(s11): evidencias finales de expiracion y matriz actualizada
</commit_message>
<xml_diff>
--- a/docs/matriz-seguridad-spa-s11.xlsx
+++ b/docs/matriz-seguridad-spa-s11.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz pruebas" sheetId="1" r:id="Rff2eb9a404bc4740"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="Re669ccf6606f40b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz pruebas" sheetId="1" r:id="Rb85001a34c7f4425"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="Rfc449fde09654b71"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -37,7 +37,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -64,11 +64,6 @@
         <x:fgColor rgb="FFFEF3C7"/>
       </x:patternFill>
     </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFEE2E2"/>
-      </x:patternFill>
-    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -77,7 +72,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="32">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -142,18 +137,6 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -927,19 +910,19 @@
         <x:v>admin</x:v>
       </x:c>
       <x:c r="D22" s="15" t="str">
-        <x:v>Configurar JWT 3 min e iniciar sesión</x:v>
+        <x:v>Configurar backend 3 minutos; probar aviso con expiraEn local a 90 s</x:v>
       </x:c>
       <x:c r="E22" s="15" t="str">
-        <x:v>Aviso aparece cuando quedan 120 s</x:v>
+        <x:v>Aviso visible cuando quedan menos de 120 s</x:v>
       </x:c>
       <x:c r="F22" s="15" t="str">
-        <x:v>Función implementada y compilada; falta prueba temporizada</x:v>
-      </x:c>
-      <x:c r="G22" s="27" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>Aviso amarillo visible a 01:08; se simuló tiempo restante en sessionStorage de navegador</x:v>
+      </x:c>
+      <x:c r="G22" s="19" t="str">
+        <x:v>PASA</x:v>
       </x:c>
       <x:c r="H22" s="15" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>B-01_aviso_mmss.png</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="74" customHeight="1">
@@ -953,19 +936,19 @@
         <x:v>admin</x:v>
       </x:c>
       <x:c r="D23" s="10" t="str">
-        <x:v>Observar contador durante 10-20 s</x:v>
+        <x:v>Observar cuenta regresiva en mm:ss</x:v>
       </x:c>
       <x:c r="E23" s="10" t="str">
-        <x:v>Cuenta regresiva cambia en mm:ss</x:v>
+        <x:v>Contador debe disminuir cada segundo</x:v>
       </x:c>
       <x:c r="F23" s="10" t="str">
-        <x:v>Sin evidencia de ejecución</x:v>
-      </x:c>
-      <x:c r="G23" s="27" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>Captura demuestra contador 01:08, pero no hay segunda captura que pruebe cambio secuencial</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="str">
+        <x:v>PARCIAL</x:v>
       </x:c>
       <x:c r="H23" s="10" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>B-02_contador_mmss.png</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="74" customHeight="1">
@@ -979,19 +962,19 @@
         <x:v>admin</x:v>
       </x:c>
       <x:c r="D24" s="15" t="str">
-        <x:v>Pulsar X en aviso y seguir sesión</x:v>
+        <x:v>Pulsar X en aviso y continuar en Inicio</x:v>
       </x:c>
       <x:c r="E24" s="15" t="str">
-        <x:v>Aviso se oculta hasta nueva sesión</x:v>
+        <x:v>Aviso se oculta sin cerrar sesión</x:v>
       </x:c>
       <x:c r="F24" s="15" t="str">
-        <x:v>Sin evidencia de ejecución</x:v>
-      </x:c>
-      <x:c r="G24" s="27" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>Se ocultó el aviso; usuario ADMIN permaneció autenticado en /inicio</x:v>
+      </x:c>
+      <x:c r="G24" s="19" t="str">
+        <x:v>PASA</x:v>
       </x:c>
       <x:c r="H24" s="15" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>B-03_ocultado.png</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="74" customHeight="1">
@@ -1005,19 +988,19 @@
         <x:v>admin</x:v>
       </x:c>
       <x:c r="D25" s="10" t="str">
-        <x:v>Dejar pasar expiración real</x:v>
+        <x:v>Simular expiración local a 15 s, recargar y observar</x:v>
       </x:c>
       <x:c r="E25" s="10" t="str">
-        <x:v>Sesión se cierra y vuelve al login</x:v>
+        <x:v>SPA vuelve automáticamente al login, con motivo y returnUrl</x:v>
       </x:c>
       <x:c r="F25" s="10" t="str">
-        <x:v>Sin evidencia de ejecución</x:v>
-      </x:c>
-      <x:c r="G25" s="27" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>Se produjo cierre de sesión con expirada=1 y returnUrl /inicio, mensaje de expiración visible</x:v>
+      </x:c>
+      <x:c r="G25" s="19" t="str">
+        <x:v>PASA</x:v>
       </x:c>
       <x:c r="H25" s="10" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>B-04_login_expirado.png</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1057,15 +1040,15 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="C2" t="n">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>1 parcial / 4 pendiente</x:v>
+        <x:v>2 parcial / 0 pendiente</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1"/>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="30" t="str">
+      <x:c r="A4" s="26" t="str">
         <x:v>Nota</x:v>
       </x:c>
       <x:c r="B4" s="8" t="str">
@@ -1073,15 +1056,15 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="30" t="str">
+      <x:c r="A5" s="26" t="str">
         <x:v>Pendientes</x:v>
       </x:c>
       <x:c r="B5" s="8" t="str">
-        <x:v>B-01 a B-04 exigen JWT con 3 minutos y capturas reales.</x:v>
+        <x:v>B-02: falta segunda medición que demuestre avance. I-01: petición externa no ejecutada.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
-      <x:c r="A6" s="30" t="str">
+      <x:c r="A6" s="26" t="str">
         <x:v>Mi cuenta</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
@@ -1089,7 +1072,7 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
-      <x:c r="A7" s="30" t="str">
+      <x:c r="A7" s="26" t="str">
         <x:v>Git</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">

</xml_diff>